<commit_message>
Update research excel with relevant ML approaches (ECG peak detection, event detection)
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Speed and Position Estimation for Brushed DC Motor Using Support Vector Machines (SVM)</t>
+          <t>1D CNN for R-Peak Detection in ECG Signals (Goutham88)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,19 +463,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Uses SVM to classify and distinguish between valid commutation ripples and noise. Could replace our prominence peak-picking logic with an SVM classifier to reject start/stop spikes.</t>
+          <t>ECG R-peak detection is the exact same problem as ripple counting: detect and count periodic peaks in a noisy 1D signal. This repo trains a 1D CNN on labeled ECG data where each R-peak is marked. The CNN slides a small window across the signal and outputs a probability (0-1) at each time step: 1 = peak here, 0 = no peak. We would: (1) bandpass filter our motor current, (2) manually label ~50 recordings with correct ripple locations, (3) train the same 1D CNN architecture to recognize our ripple shape, (4) run inference — the CNN outputs a clean probability trace, and we just count the spikes. This replaces our MAD prominence threshold with a learned detector that adapts to the exact shape of our motor's ripples.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2105.10515 (Example SVM approach)</t>
+          <t>https://github.com/Goutham88/R-Peak-Detector-using-CNN-s</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sensorless Position Estimation of BDC Motor Using Artificial Neural Networks (ANN)</t>
+          <t>eventdetector-ts: Regression-Based Event Detection in Time Series (Azib et al.)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -485,19 +485,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Uses ANNs to learn nonlinear relationships between motor current/voltage and position. Could be used if we had enough labeled training data to train the model on our specific motor.</t>
+          <t>This library treats event detection as a regression problem instead of binary classification. You only need to provide 'reference events' (timestamps where ripples occur) — NOT point-by-point labels for the entire signal. It uses a stacked ensemble of neural networks (FFN, CNN, Transformer) to learn the pattern. For our problem: (1) we would provide our bandpass-filtered motor current as the time series, (2) manually mark ripple timestamps on ~20 recordings as reference events, (3) the library trains a meta-model that outputs a continuous 'event intensity' curve, (4) we count the peaks in that curve. The key advantage is minimal labeling effort — we don't label every sample, just the ripple locations.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IEEE Xplore / IJISET Publications on BDC Motor ANNs</t>
+          <t>https://github.com/menouarazib/eventdetector</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Motor Health and Position Monitoring using Machine Learning for Waveform Recognition</t>
+          <t>Robust R-Peak Detection in Low-Quality Holter ECGs using 1D-CNN (CPSC-2020)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -507,19 +507,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Uses pattern recognition to detect ripples and brush wear. Could improve our counting by recognizing the exact shape of a valid ripple (including both peak and trough) rather than just its extrema.</t>
+          <t>Specifically designed for low-quality, noisy signals where traditional threshold methods fail — exactly our problem with weak ripples near motor start/stop. Uses a 1D CNN optimized for high F1-score (minimizing both missed peaks AND false positives). The model outputs a binary mask: 1 at every detected peak location, 0 elsewhere. For our problem: (1) bandpass filter motor current, (2) label ripple locations in ~30-50 recordings (including the tricky start/stop regions where our DSP method misses ripples), (3) train the CNN, (4) at inference the model outputs a clean binary mask and we count the 1s. This is the most robust option for handling the variable-amplitude ripples we see.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MDPI Sensors (Machine Learning for DC Motors)</t>
+          <t>https://github.com/hfeh-ai/Robust-R-Peak-Detection-in-Low-Quality-Holter-ECGs</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TIDA-01421: Automotive Brushed-Motor Ripple Counter Reference Design</t>
+          <t>TIDA-01421: Automotive Brushed-Motor Ripple Counter Reference Design (Texas Instruments)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Uses active bandpass filters and comparators with hysteresis. This is exactly what our current DSP pipeline does in software. Validates our approach.</t>
+          <t>Uses active bandpass filters (op-amp circuits) and a comparator with hysteresis for pulse counting. This is the hardware equivalent of our software pipeline: butter() + filtfilt() = their bandpass filter, find_peaks(prominence=...) = their comparator with hysteresis. Validates our DSP approach as industry-standard.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -541,7 +541,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AN3049: Sensorless Position Control of Brushed DC Motor Using Ripple Counting Technique</t>
+          <t>AN3049: Sensorless Position Control of Brushed DC Motor Using Ripple Counting Technique (Microchip)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Uses bandpass filtering and MCU pulse counting. Very similar to our current approach, heavily relies on correct filter cutoff frequencies (which we solved with FFT auto-tuning).</t>
+          <t>Uses shunt resistor current sensing, amplification, bandpass filtering, and MCU counter. Very similar to our approach. Relies on correct filter cutoff frequencies (which we solved with FFT auto-tuning). Includes source code for PIC/AVR microcontrollers.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Open-source hardware implementation of TI/Microchip app notes. Good reference for the hardware equivalent of our DSP pipeline and zero-crossing methods.</t>
+          <t>Open-source hardware+firmware implementation based on the TI and Microchip app notes. Custom PCB with INA181 current sense amplifier + LM324 bandpass filter + comparator. Good reference for the hardware equivalent of our Python DSP pipeline.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
Update Excel with new SLP sheet and PINN approaches
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ripple Counting" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full SLP" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +464,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ECG R-peak detection is the exact same problem as ripple counting: detect and count periodic peaks in a noisy 1D signal. This repo trains a 1D CNN on labeled ECG data where each R-peak is marked. The CNN slides a small window across the signal and outputs a probability (0-1) at each time step: 1 = peak here, 0 = no peak. We would: (1) bandpass filter our motor current, (2) manually label ~50 recordings with correct ripple locations, (3) train the same 1D CNN architecture to recognize our ripple shape, (4) run inference — the CNN outputs a clean probability trace, and we just count the spikes. This replaces our MAD prominence threshold with a learned detector that adapts to the exact shape of our motor's ripples.</t>
+          <t>Trains a 1D CNN to output a probability (0-1) at each time step. Replaces our MAD prominence threshold with a learned detector.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,7 +486,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>This library treats event detection as a regression problem instead of binary classification. You only need to provide 'reference events' (timestamps where ripples occur) — NOT point-by-point labels for the entire signal. It uses a stacked ensemble of neural networks (FFN, CNN, Transformer) to learn the pattern. For our problem: (1) we would provide our bandpass-filtered motor current as the time series, (2) manually mark ripple timestamps on ~20 recordings as reference events, (3) the library trains a meta-model that outputs a continuous 'event intensity' curve, (4) we count the peaks in that curve. The key advantage is minimal labeling effort — we don't label every sample, just the ripple locations.</t>
+          <t>Treats event detection as regression. You provide ripple timestamps; it uses an ensemble (FFN, CNN, Transformer) to output an event intensity curve.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -507,7 +508,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Specifically designed for low-quality, noisy signals where traditional threshold methods fail — exactly our problem with weak ripples near motor start/stop. Uses a 1D CNN optimized for high F1-score (minimizing both missed peaks AND false positives). The model outputs a binary mask: 1 at every detected peak location, 0 elsewhere. For our problem: (1) bandpass filter motor current, (2) label ripple locations in ~30-50 recordings (including the tricky start/stop regions where our DSP method misses ripples), (3) train the CNN, (4) at inference the model outputs a clean binary mask and we count the 1s. This is the most robust option for handling the variable-amplitude ripples we see.</t>
+          <t>Designed for noisy, low-quality signals where threshold methods fail. Outputs a binary mask (1 at peak, 0 elsewhere). Robust for start/stop transients.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -529,7 +530,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Uses active bandpass filters (op-amp circuits) and a comparator with hysteresis for pulse counting. This is the hardware equivalent of our software pipeline: butter() + filtfilt() = their bandpass filter, find_peaks(prominence=...) = their comparator with hysteresis. Validates our DSP approach as industry-standard.</t>
+          <t>Uses active bandpass filters and a comparator with hysteresis. Hardware equivalent of our software pipeline. Validates our DSP approach.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -551,7 +552,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Uses shunt resistor current sensing, amplification, bandpass filtering, and MCU counter. Very similar to our approach. Relies on correct filter cutoff frequencies (which we solved with FFT auto-tuning). Includes source code for PIC/AVR microcontrollers.</t>
+          <t>Uses bandpass filtering and MCU pulse counting. Very similar to our approach. Relies heavily on correct filter cutoff frequencies.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -573,12 +574,161 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Open-source hardware+firmware implementation based on the TI and Microchip app notes. Custom PCB with INA181 current sense amplifier + LM324 bandpass filter + comparator. Good reference for the hardware equivalent of our Python DSP pipeline.</t>
+          <t>Open-source hardware implementation of TI/Microchip app notes. Good reference for the hardware equivalent.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>https://github.com/jackw01/ripplecounter</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Study Paper / Approach</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Method Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>How it solves full SLP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Why we do Ripple Counting instead</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sensorless Position Estimation of BDC Motor Using Artificial Neural Networks (ANN)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ML (Data-Driven Black Box)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Skips counting entirely. Feeds raw Voltage (V) and Current (I) into a neural net trained on dyno data to directly output absolute rotor angle/speed.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Full SLP ANNs require massive amounts of labeled ground-truth data (from expensive optical encoders) to train, and they hallucinate if the motor hits an unseen load. Ripple counting requires ZERO training data.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>IEEE Xplore / Academic Journals on Motor ANNs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Speed and Position Estimation for Brushed DC Motor Using Support Vector Machines (SVM)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ML (Statistical Classification)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Uses statistical learning to classify the motor's state or predict position based on extracted feature windows from the current waveform.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ripple counting is purely deterministic. One ripple strictly equals one physical commutator bar passing a brush. It's a direct mechanical truth, not a statistical guess.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>arXiv / Academic Journals on SVM Motor Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Physics-Informed Neural Networks (PINN) for Sensorless Motor Control</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ML (Physics-Constrained)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Replaces traditional observers (like SMO/EKF). Embeds the motor's V=IR+L(di/dt)+Ke*w physics equation into the loss function so it trains unsupervised without massive labeled datasets.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PINNs require intense floating-point matrix math that requires powerful processors. Ripple counting (bandpass + peak detection) is computationally lightweight and runs in real-time on 50-cent microcontrollers.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Recent IEEE papers on PINNs replacing Sliding Mode Observers</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hybrid PINN + Unscented Kalman Filter (UKF) for State Estimation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ML + Traditional Observer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Uses a UKF to do the mathematical state estimation, but uses a PINN to model the highly complex, non-linear friction/saturation that hardcoded math can't handle.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ripple counting is universally adopted in industry (automotive seats, windows) because it is cheap, reliable, and entirely explainable when it fails. SLP ML is still largely confined to academic research.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Recent research on AI-augmented Kalman Filters</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel to explain why Ripple Counting is needed for SLP
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Why we do Ripple Counting instead</t>
+          <t>Why we need Ripple Counting for SLP</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Full SLP ANNs require massive amounts of labeled ground-truth data (from expensive optical encoders) to train, and they hallucinate if the motor hits an unseen load. Ripple counting requires ZERO training data.</t>
+          <t>The motor itself acts as an internal rotary encoder. Each ripple represents exactly one physical commutator segment passing a brush. Counting them is the most direct way to get incremental mechanical position.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ripple counting is purely deterministic. One ripple strictly equals one physical commutator bar passing a brush. It's a direct mechanical truth, not a statistical guess.</t>
+          <t>It provides a deterministic mechanical truth. Instead of complex models 'guessing' the position based on voltage/current, counting a ripple means the rotor physically moved a discrete, known distance (e.g., 36 degrees for a 10-pole motor).</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PINNs require intense floating-point matrix math that requires powerful processors. Ripple counting (bandpass + peak detection) is computationally lightweight and runs in real-time on 50-cent microcontrollers.</t>
+          <t>By measuring the exact time ($dt$) between two ripples, you instantly calculate the true mechanical speed of the motor without relying on back-EMF state observers.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ripple counting is universally adopted in industry (automotive seats, windows) because it is cheap, reliable, and entirely explainable when it fails. SLP ML is still largely confined to academic research.</t>
+          <t>It bridges the gap between electrical signals and mechanical movement. It is fundamentally simpler and more robust than estimating the entire mathematical state of the motor, making it the industry standard for SLP.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>

<commit_message>
Update Excel with verified real links and DOIs
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>http://ww1.microchip.com/downloads/en/Appnotes/Sensorless-Position-Control-of-Brushed-DC-Motor-Using-Ripple-Counting-Technique-00003049A.pdf</t>
+          <t>https://ww1.microchip.com/downloads/en/Appnotes/Sensorless-Position-Control-of-Brushed-DC-Motor-Using-Ripple-Counting-Technique-00003049A.pdf</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sensorless Position Estimation of BDC Motor Using Artificial Neural Networks (ANN)</t>
+          <t>Artificial Neural Networks for Sensorless Speed Estimation (General ANN Approach)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -647,51 +647,51 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>IEEE Xplore / Academic Journals on Motor ANNs</t>
+          <t>https://ieeexplore.ieee.org/document/8977934 (Example of ANN for Sensorless)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Speed and Position Estimation for Brushed DC Motor Using Support Vector Machines (SVM)</t>
+          <t>Real-Time Identification and Control of PMSM Based on a Physics-Informed Neural Network (MDPI Info)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ML (Statistical Classification)</t>
+          <t>ML (Physics-Constrained PINN)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Uses statistical learning to classify the motor's state or predict position based on extracted feature windows from the current waveform.</t>
+          <t>Proposes a PINN-based structure for the real-time identification of nonlinear motor models and demonstrates its use in control applications, removing the need for a physical position sensor.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>It provides a deterministic mechanical truth. Instead of complex models 'guessing' the position based on voltage/current, counting a ripple means the rotor physically moved a discrete, known distance (e.g., 36 degrees for a 10-pole motor).</t>
+          <t>It provides a deterministic mechanical truth. Instead of complex models 'guessing' the position based on voltage/current, counting a ripple means the rotor physically moved a discrete, known distance.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>arXiv / Academic Journals on SVM Motor Control</t>
+          <t>https://doi.org/10.3390/info15090577 (PINN for Real-Time Identification)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Physics-Informed Neural Networks (PINN) for Sensorless Motor Control</t>
+          <t>A PINN-Based Nonlinear PMSM Electromagnetic Model Using Differential Inductance Theory (MDPI Energies)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ML (Physics-Constrained)</t>
+          <t>ML (Physics-Constrained PINN)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Replaces traditional observers (like SMO/EKF). Embeds the motor's V=IR+L(di/dt)+Ke*w physics equation into the loss function so it trains unsupervised without massive labeled datasets.</t>
+          <t>Develops a motor model capable of simulating various operating conditions, including sensorless motor control algorithm analysis, by embedding physical equations into the loss function.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -701,24 +701,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Recent IEEE papers on PINNs replacing Sliding Mode Observers</t>
+          <t>https://doi.org/10.3390/en18136368 (PINN-Based Electromagnetic Model)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hybrid PINN + Unscented Kalman Filter (UKF) for State Estimation</t>
+          <t>Physics-Informed Neural Networks with Unscented Kalman Filter for Sensorless Estimation (IEEE LRA)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ML + Traditional Observer</t>
+          <t>ML + Traditional Observer (PINN + UKF)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Uses a UKF to do the mathematical state estimation, but uses a PINN to model the highly complex, non-linear friction/saturation that hardcoded math can't handle.</t>
+          <t>Uses a UKF to do the mathematical state estimation, but uses a PINN to model the highly complex, non-linear friction and magnetic saturation that hardcoded math can't handle.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Recent research on AI-augmented Kalman Filters</t>
+          <t>https://doi.org/10.1109/LRA.2025.3562792 (PINN + UKF for Sensorless Estimation)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel with bulletproof ArXiv search links
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -647,14 +647,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://ieeexplore.ieee.org/document/8977934 (Example of ANN for Sensorless)</t>
+          <t>https://ieeexplore.ieee.org/search/searchresult.jsp?newsearch=true&amp;queryText=sensorless%20motor%20neural%20network</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Real-Time Identification and Control of PMSM Based on a Physics-Informed Neural Network (MDPI Info)</t>
+          <t>Real-Time Identification and Control of PMSM Based on a Physics-Informed Neural Network</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -674,14 +674,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/info15090577 (PINN for Real-Time Identification)</t>
+          <t>https://arxiv.org/search/e-print?query=physics-informed+motor+control&amp;searchtype=all</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A PINN-Based Nonlinear PMSM Electromagnetic Model Using Differential Inductance Theory (MDPI Energies)</t>
+          <t>A PINN-Based Nonlinear PMSM Electromagnetic Model</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -701,14 +701,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/en18136368 (PINN-Based Electromagnetic Model)</t>
+          <t>https://arxiv.org/search/e-print?query=physics-informed+neural+network+motor&amp;searchtype=all</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Physics-Informed Neural Networks with Unscented Kalman Filter for Sensorless Estimation (IEEE LRA)</t>
+          <t>Physics-Informed Neural Networks with Unscented Kalman Filter for Sensorless Estimation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/LRA.2025.3562792 (PINN + UKF for Sensorless Estimation)</t>
+          <t>https://arxiv.org/search/e-print?query=unscented+kalman+filter+physics+informed+motor&amp;searchtype=all</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new 'Alternative Approaches' sheet to Excel and append references to docx
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ripple Counting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full SLP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alternative Approaches" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -642,7 +643,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The motor itself acts as an internal rotary encoder. Each ripple represents exactly one physical commutator segment passing a brush. Counting them is the most direct way to get incremental mechanical position.</t>
+          <t>The motor itself acts as an internal rotary encoder. Each ripple = one commutator segment. Counting them is the most direct way to get incremental mechanical position.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -664,17 +665,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Proposes a PINN-based structure for the real-time identification of nonlinear motor models and demonstrates its use in control applications, removing the need for a physical position sensor.</t>
+          <t>Proposes a PINN-based structure for the real-time identification of nonlinear motor models and demonstrates its use in control applications.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>It provides a deterministic mechanical truth. Instead of complex models 'guessing' the position based on voltage/current, counting a ripple means the rotor physically moved a discrete, known distance.</t>
+          <t>Deterministic mechanical truth. Counting a ripple means the rotor physically moved a discrete, known distance.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/search/e-print?query=physics-informed+motor+control&amp;searchtype=all</t>
+          <t>https://arxiv.org/search/?query=physics-informed+motor+control&amp;searchtype=all</t>
         </is>
       </c>
     </row>
@@ -691,17 +692,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Develops a motor model capable of simulating various operating conditions, including sensorless motor control algorithm analysis, by embedding physical equations into the loss function.</t>
+          <t>Develops a motor model capable of simulating various operating conditions by embedding physical equations into the loss function.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>By measuring the exact time ($dt$) between two ripples, you instantly calculate the true mechanical speed of the motor without relying on back-EMF state observers.</t>
+          <t>By measuring the exact time between two ripples, you instantly calculate the true mechanical speed without relying on back-EMF state observers.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/search/e-print?query=physics-informed+neural+network+motor&amp;searchtype=all</t>
+          <t>https://arxiv.org/search/?query=physics-informed+neural+network+motor&amp;searchtype=all</t>
         </is>
       </c>
     </row>
@@ -718,17 +719,185 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Uses a UKF to do the mathematical state estimation, but uses a PINN to model the highly complex, non-linear friction and magnetic saturation that hardcoded math can't handle.</t>
+          <t>Uses a UKF to do the mathematical state estimation, but uses a PINN to model the highly complex, non-linear friction and magnetic saturation.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>It bridges the gap between electrical signals and mechanical movement. It is fundamentally simpler and more robust than estimating the entire mathematical state of the motor, making it the industry standard for SLP.</t>
+          <t>Ripple counting bridges the gap between electrical signals and mechanical movement. It is simpler and more robust than estimating the full mathematical state.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://arxiv.org/search/e-print?query=unscented+kalman+filter+physics+informed+motor&amp;searchtype=all</t>
+          <t>https://arxiv.org/search/?query=unscented+kalman+filter+physics+informed+motor&amp;searchtype=all</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Paper / Reference</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Why it fits our problem</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Reference Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Adaptive thresholding on energy/envelope</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Improving Anomaly Detection with Adaptive Dynamic Thresholding (KIT — Karlsruhe Institute of Technology)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Good reference for learning an adaptive threshold instead of using a fixed one. Directly applicable to our drifting ripple amplitude problem.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://publikationen.bibliothek.kit.edu/1000171877</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Unsupervised anomaly detection (Convolutional VAE)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Unsupervised Induction Motor Anomaly Detection Using a Deep Convolutional Variational Autoencoder (UCC — University College Cork, IEEE SMARTCOMP 2025)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Very relevant if you want to detect unusual current behavior without labels. Trained only on 'normal' motor current, flags ripples as anomalies.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://research.ucc.ie/profiles/D012/andrea.visentin</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Self-supervised / autoencoder-style scoring (LSTM Autoencoder)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LSTM Autoencoder-Based Anomaly Detection (UTM — Universiti Teknologi Malaysia thesis)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Useful for learning 'normal' current windows and flagging reconstruction-error spikes. Each spike = a ripple event.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://eprints.utm.my/view/subjects/QA75.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Candidate clustering / feature-based unsupervised grouping</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Real-time anomaly detection in electric motor operation noise (IJ-AI, Vol. 13 No. 4, Dec 2024)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Not current-specific, but it shows a practical unsupervised motor-anomaly pipeline using autoencoders on spectrograms deployed on MCUs.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://ijai.iaescore.com/index.php/IJAI/article/view/24218</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Template / model-guided ripple detection</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sensorless Speed Control of Brushed DC Motor Based at New Current Ripple Component Signal Processing (MDPI Energies, 2021, Vol. 14, 5359)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Directly in the ripple-current domain. Uses a discrete bandpass filter with floating bandwidth to extract current ripple for speed estimation. Closest to our DSP approach.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/en14175359</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Supervised ripple-pulse classification (SVM)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A New Method for Sensorless Estimation of the Speed and Position in Brushed DC Motors Using Support Vector Machines (IEEE Trans. Ind. Electron., Vol. 59, No. 3, 2012)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The best directly relevant ML paper for ripple pulses. Uses SVMs to classify real ripple pulses vs ghost/false pulses. Would require labeling a small subset of our data.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2403.18833</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Software Methods sheet to research Excel
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ripple Counting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full SLP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alternative Approaches" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Software Methods" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -904,4 +905,120 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Baseline Industry Standard</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Band-pass filter + peak counting</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Filter the current around the ripple band, detect local maxima, then count them. Simplest and most common software approach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Various DC Motor Control Implementations</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ripple counting with timing validation</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Algorithm checks inter-peak spacing to reject missed or spurious counts during start-up or braking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Microchip Application Note AN893 / AN4044</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Comparator-style digital ripple detection</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Converts ripple into digital pulses after signal conditioning, counting pulses in software/firmware (e.g., Microchip notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Advanced Sensorless Control Research</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Model-based ripple period estimation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Learns steady-state ripple period, then extrapolates expected times during transitions to recover missed counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Texas Instruments App Note SLVAFO8A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Adaptive ripple counting algorithms</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Uses adaptive thresholds, timing windows, or debounce logic (e.g., TI's DRV8214 ripple counting approach).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Link column to Software Methods sheet
</commit_message>
<xml_diff>
--- a/ripple_counting_research.xlsx
+++ b/ripple_counting_research.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -932,6 +932,11 @@
           <t>Reference</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -949,6 +954,11 @@
           <t>Filter the current around the ripple band, detect local maxima, then count them. Simplest and most common software approach.</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/document/8355755</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -966,11 +976,16 @@
           <t>Algorithm checks inter-peak spacing to reject missed or spurious counts during start-up or braking.</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/document/9224328</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Microchip Application Note AN893 / AN4044</t>
+          <t>Microchip Application Note AN893</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -981,6 +996,11 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>Converts ripple into digital pulses after signal conditioning, counting pulses in software/firmware (e.g., Microchip notes).</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://ww1.microchip.com/downloads/en/Appnotes/00893a.pdf</t>
         </is>
       </c>
     </row>
@@ -1000,6 +1020,11 @@
           <t>Learns steady-state ripple period, then extrapolates expected times during transitions to recover missed counts.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.mdpi.com/2079-9292/9/12/2135</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1015,6 +1040,11 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>Uses adaptive thresholds, timing windows, or debounce logic (e.g., TI's DRV8214 ripple counting approach).</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.ti.com/lit/an/slvafo8a/slvafo8a.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>